<commit_message>
Update dataset evaluation to use local Postgres and improve agent behavior
- Replace task_reminder.py with dataset_evaluation.py that runs tests against local Postgres
- Add scratchpad intermediate writes so partial results are visible on think() timeout
- Add elapsed_s timing to scratchpad entries
- Update system prompt: tie 'one moment' acknowledgment to actual tool call
- Change duplicate tool call response from verbose [COMPLETED] to [SILENT_NO_RESPONSE_NEEDED] to prevent hallucination
- Add README for integration test setup

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/test/integration/test_inputs.xlsx
+++ b/test/integration/test_inputs.xlsx
@@ -12,13 +12,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,11 +44,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,11 +452,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,6 +483,21 @@
           <t>Scratchpad</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Setup Query</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>DB State Before</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>DB State After</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -503,19 +525,72 @@
   },
   {
     "source": "agent",
+    "format": "audio",
+    "content": "One moment."
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "create_tasks_tool",
+    "response": {
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'take my medicine'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"a5594cdb-d0bd-47d5-b164-dbaf9ae70df3\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T23:00:00-08:00\"}"
+    },
+    "elapsed_s": 13.27
+  },
+  {
+    "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-6405358909444243832",
+    "call_id": "function-call-2218109440114766425",
     "response": {
       "result": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
-    }
+    },
+    "elapsed_s": 0.0
   },
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment. Of course! I've set a reminder to take your medicine at 11:00 PM today."
+    "content": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]: (empty)
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | True
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+a5594cdb-d0bd-47d5-b164-dbaf9ae70df3 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 23:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>
@@ -532,7 +607,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment, let me check.</t>
+          <t>AGENT: One moment, let me check. Idaho You have one task today: take my medicine at 12:00 PM today.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -546,9 +621,74 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment, let me check."
+    "content": "One moment, let me check. Idaho"
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "get_tasks_tool",
+    "response": {
+      "result": "{\"tasks\": [{\"task_id\": \"e73a8438-a468-4557-9139-26b3b1479fea\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
+    },
+    "elapsed_s": 12.57
+  },
+  {
+    "source": "agent",
+    "format": "function_call",
+    "name": "think_and_repeat_output",
+    "call_id": "function-call-15670564726536839728",
+    "response": {
+      "result": "\n\nYou have one task today:\n- Take my medicine at 12:00 PM today."
+    },
+    "elapsed_s": 0.0
+  },
+  {
+    "source": "agent",
+    "format": "audio",
+    "content": "You have one task today: take my medicine at 12:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING; INSERT INTO tasks (task_id, user_id, task_info, status, time_to_execute) VALUES (gen_random_uuid(), '2ba330c0-a999-46f8-ba2c-855880bdcf5b', '{"info": "take my medicine"}', 'pending', '2026-03-01T12:00:00-08:00')</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>
@@ -565,7 +705,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment,</t>
+          <t>AGENT: One moment. I've set a reminder to stretch at 10:00 PM today.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -579,9 +719,71 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment,"
+    "content": "One moment."
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "create_tasks_tool",
+    "response": {
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'strecth'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"7a9f7b2b-2b98-44f6-8c1b-50d886268528\", \"task_info\": {\"info\": \"strecth\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T22:00:00-08:00\"}"
+    },
+    "elapsed_s": 11.63
+  },
+  {
+    "source": "agent",
+    "format": "function_call",
+    "name": "think_and_repeat_output",
+    "call_id": "function-call-3680642655420553762",
+    "response": {
+      "result": "I've set a reminder to strecth at 10:00 PM today."
+    },
+    "elapsed_s": 0.0
+  },
+  {
+    "source": "agent",
+    "format": "audio",
+    "content": "I've set a reminder to stretch at 10:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]: (empty)
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+7a9f7b2b-2b98-44f6-8c1b-50d886268528 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'strecth'} | pending | 2026-03-01 22:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dataset evaluation to use local Postgres and improve agent behavior (#54)
- Replace task_reminder.py with dataset_evaluation.py that runs tests against local Postgres
- Add scratchpad intermediate writes so partial results are visible on think() timeout
- Add elapsed_s timing to scratchpad entries
- Update system prompt: tie 'one moment' acknowledgment to actual tool call
- Change duplicate tool call response from verbose [COMPLETED] to [SILENT_NO_RESPONSE_NEEDED] to prevent hallucination
- Add README for integration test setup

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/test/integration/test_inputs.xlsx
+++ b/test/integration/test_inputs.xlsx
@@ -12,13 +12,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,11 +44,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,11 +452,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -476,6 +483,21 @@
           <t>Scratchpad</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Setup Query</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>DB State Before</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>DB State After</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -503,19 +525,72 @@
   },
   {
     "source": "agent",
+    "format": "audio",
+    "content": "One moment."
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "create_tasks_tool",
+    "response": {
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'take my medicine'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"a5594cdb-d0bd-47d5-b164-dbaf9ae70df3\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T23:00:00-08:00\"}"
+    },
+    "elapsed_s": 13.27
+  },
+  {
+    "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-6405358909444243832",
+    "call_id": "function-call-2218109440114766425",
     "response": {
       "result": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
-    }
+    },
+    "elapsed_s": 0.0
   },
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment. Of course! I've set a reminder to take your medicine at 11:00 PM today."
+    "content": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]: (empty)
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | True
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+a5594cdb-d0bd-47d5-b164-dbaf9ae70df3 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 23:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>
@@ -532,7 +607,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment, let me check.</t>
+          <t>AGENT: One moment, let me check. Idaho You have one task today: take my medicine at 12:00 PM today.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -546,9 +621,74 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment, let me check."
+    "content": "One moment, let me check. Idaho"
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "get_tasks_tool",
+    "response": {
+      "result": "{\"tasks\": [{\"task_id\": \"e73a8438-a468-4557-9139-26b3b1479fea\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
+    },
+    "elapsed_s": 12.57
+  },
+  {
+    "source": "agent",
+    "format": "function_call",
+    "name": "think_and_repeat_output",
+    "call_id": "function-call-15670564726536839728",
+    "response": {
+      "result": "\n\nYou have one task today:\n- Take my medicine at 12:00 PM today."
+    },
+    "elapsed_s": 0.0
+  },
+  {
+    "source": "agent",
+    "format": "audio",
+    "content": "You have one task today: take my medicine at 12:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING; INSERT INTO tasks (task_id, user_id, task_info, status, time_to_execute) VALUES (gen_random_uuid(), '2ba330c0-a999-46f8-ba2c-855880bdcf5b', '{"info": "take my medicine"}', 'pending', '2026-03-01T12:00:00-08:00')</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>
@@ -565,7 +705,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment,</t>
+          <t>AGENT: One moment. I've set a reminder to stretch at 10:00 PM today.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -579,9 +719,71 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment,"
+    "content": "One moment."
+  },
+  {
+    "source": "agent_internal",
+    "format": "function_call",
+    "name": "create_tasks_tool",
+    "response": {
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'strecth'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"7a9f7b2b-2b98-44f6-8c1b-50d886268528\", \"task_info\": {\"info\": \"strecth\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T22:00:00-08:00\"}"
+    },
+    "elapsed_s": 11.63
+  },
+  {
+    "source": "agent",
+    "format": "function_call",
+    "name": "think_and_repeat_output",
+    "call_id": "function-call-3680642655420553762",
+    "response": {
+      "result": "I've set a reminder to strecth at 10:00 PM today."
+    },
+    "elapsed_s": 0.0
+  },
+  {
+    "source": "agent",
+    "format": "audio",
+    "content": "I've set a reminder to stretch at 10:00 PM today."
   }
 ]</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>INSERT INTO users (user_id, first_name, last_name, timezone) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', 'Grandma', NULL, 'America/Los_Angeles') ON CONFLICT (user_id) DO NOTHING; INSERT INTO sessions (user_id, scratchpad, is_active) VALUES ('2ba330c0-a999-46f8-ba2c-855880bdcf5b', '', false) ON CONFLICT (user_id) DO NOTHING</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]: (empty)
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>[users]:
+user_id | first_name | last_name | firebase_uid | username | timezone | device_prefix
+-------------------------------------------------------------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b | Grandma | None | None | None | America/Los_Angeles | None
+[sessions]:
+user_id | scratchpad | is_active
+--------------------------------
+2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
+[tasks]:
+task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
+------------------------------------------------------------------------------
+7a9f7b2b-2b98-44f6-8c1b-50d886268528 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'strecth'} | pending | 2026-03-01 22:00:00-08:00 | None
+[messages]: (empty)
+[pending_text_message_jobs]: (empty)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Setup integration test for windows
</commit_message>
<xml_diff>
--- a/test/integration/test_inputs.xlsx
+++ b/test/integration/test_inputs.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment. Of course! I've set a reminder to take your medicine at 11:00 PM today.</t>
+          <t>AGENT: One moment, I've set a reminder to take your medicine at 11:00 PM today.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -526,31 +526,31 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment."
+    "content": "One moment,"
   },
   {
     "source": "agent_internal",
     "format": "function_call",
     "name": "create_tasks_tool",
     "response": {
-      "result": "{\"success\": true, \"message\": \"Task '{'info': 'take my medicine'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"a5594cdb-d0bd-47d5-b164-dbaf9ae70df3\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T23:00:00-08:00\"}"
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'take my medicine'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"635e6bfc-25a8-49f2-beec-1359737efc67\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T23:00:00-08:00\", \"enqueue_result\": {\"success\": true, \"task_id\": \"635e6bfc-25a8-49f2-beec-1359737efc67\", \"scheduled_time\": \"2026-03-02T07:00:00+00:00\", \"message\": \"Task scheduled for 2026-03-02 07:00:00 UTC\", \"sequence_id\": 648}}"
     },
-    "elapsed_s": 13.27
+    "elapsed_s": 14.56
   },
   {
     "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-2218109440114766425",
+    "call_id": "function-call-3891876598665255758",
     "response": {
-      "result": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
+      "result": "I've set a reminder to take your medicine at 11:00 PM today."
     },
     "elapsed_s": 0.0
   },
   {
     "source": "agent",
     "format": "audio",
-    "content": "Of course! I've set a reminder to take your medicine at 11:00 PM today."
+    "content": "I've set a reminder to take your medicine at 11:00 PM today."
   }
 ]</t>
         </is>
@@ -588,7 +588,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-a5594cdb-d0bd-47d5-b164-dbaf9ae70df3 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 23:00:00-08:00 | None
+635e6bfc-25a8-49f2-beec-1359737efc67 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 23:00:00-08:00 | 648
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -607,7 +607,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment, let me check. Idaho You have one task today: take my medicine at 12:00 PM today.</t>
+          <t>AGENT: Let me check. You have one task scheduled for today: Take my medicine at 12:00 PM today.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -621,31 +621,31 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment, let me check. Idaho"
+    "content": "Let me check."
   },
   {
     "source": "agent_internal",
     "format": "function_call",
     "name": "get_tasks_tool",
     "response": {
-      "result": "{\"tasks\": [{\"task_id\": \"e73a8438-a468-4557-9139-26b3b1479fea\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
+      "result": "{\"tasks\": [{\"task_id\": \"4f76c3a7-a4dd-4dc7-92e2-60ec181a19ec\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
     },
-    "elapsed_s": 12.57
+    "elapsed_s": 13.47
   },
   {
     "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-15670564726536839728",
+    "call_id": "function-call-4240552157724820194",
     "response": {
-      "result": "\n\nYou have one task today:\n- Take my medicine at 12:00 PM today."
+      "result": "You have one task scheduled for today: \n- Take my medicine at 12:00 PM today."
     },
     "elapsed_s": 0.0
   },
   {
     "source": "agent",
     "format": "audio",
-    "content": "You have one task today: take my medicine at 12:00 PM today."
+    "content": "You have one task scheduled for today: Take my medicine at 12:00 PM today."
   }
 ]</t>
         </is>
@@ -668,7 +668,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+4f76c3a7-a4dd-4dc7-92e2-60ec181a19ec | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -686,7 +686,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-e73a8438-a468-4557-9139-26b3b1479fea | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+4f76c3a7-a4dd-4dc7-92e2-60ec181a19ec | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -705,7 +705,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment. I've set a reminder to stretch at 10:00 PM today.</t>
+          <t>AGENT: One moment, let me set that for you.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -719,31 +719,7 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment."
-  },
-  {
-    "source": "agent_internal",
-    "format": "function_call",
-    "name": "create_tasks_tool",
-    "response": {
-      "result": "{\"success\": true, \"message\": \"Task '{'info': 'strecth'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"7a9f7b2b-2b98-44f6-8c1b-50d886268528\", \"task_info\": {\"info\": \"strecth\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T22:00:00-08:00\"}"
-    },
-    "elapsed_s": 11.63
-  },
-  {
-    "source": "agent",
-    "format": "function_call",
-    "name": "think_and_repeat_output",
-    "call_id": "function-call-3680642655420553762",
-    "response": {
-      "result": "I've set a reminder to strecth at 10:00 PM today."
-    },
-    "elapsed_s": 0.0
-  },
-  {
-    "source": "agent",
-    "format": "audio",
-    "content": "I've set a reminder to stretch at 10:00 PM today."
+    "content": "One moment, let me set that for you."
   }
 ]</t>
         </is>
@@ -778,10 +754,7 @@
 user_id | scratchpad | is_active
 --------------------------------
 2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | False
-[tasks]:
-task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
-------------------------------------------------------------------------------
-7a9f7b2b-2b98-44f6-8c1b-50d886268528 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'strecth'} | pending | 2026-03-01 22:00:00-08:00 | None
+[tasks]: (empty)
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>

</xml_diff>

<commit_message>
Long overdue updates: Tests handle compressed audio from server. Updated integration test setup. Switched to lates live api model.
</commit_message>
<xml_diff>
--- a/test/integration/test_inputs.xlsx
+++ b/test/integration/test_inputs.xlsx
@@ -512,7 +512,7 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment, let me set that for you. I've set a reminder for you to take your medicine at 11:00 PM today.</t>
+          <t>AGENT: One moment.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -526,31 +526,7 @@
   {
     "source": "agent",
     "format": "audio",
-    "content": "One moment, let me set that for you."
-  },
-  {
-    "source": "agent_internal",
-    "format": "function_call",
-    "name": "create_tasks_tool",
-    "response": {
-      "result": "{\"success\": true, \"message\": \"Task '{'info': 'take my medicine'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"091178a2-b1e0-487f-bd6f-97754d2ab2e5\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T23:00:00-08:00\"}"
-    },
-    "elapsed_s": 12.75
-  },
-  {
-    "source": "agent",
-    "format": "function_call",
-    "name": "think_and_repeat_output",
-    "call_id": "function-call-13718634867651651649",
-    "response": {
-      "result": "\n\nI've set a reminder for you to take your medicine at 11:00 PM today."
-    },
-    "elapsed_s": 0.0
-  },
-  {
-    "source": "agent",
-    "format": "audio",
-    "content": "I've set a reminder for you to take your medicine at 11:00 PM today."
+    "content": "One moment."
   }
 ]</t>
         </is>
@@ -585,10 +561,7 @@
 user_id | scratchpad | is_active
 --------------------------------
 2ba330c0-a999-46f8-ba2c-855880bdcf5b |  | True
-[tasks]:
-task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
-------------------------------------------------------------------------------
-091178a2-b1e0-487f-bd6f-97754d2ab2e5 | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 23:00:00-08:00 | None
+[tasks]: (empty)
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -607,7 +580,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment, let me check your tasks. You have one task scheduled for today: take your medicine at 12:00 PM.</t>
+          <t>AGENT: You have one task scheduled for today: take your medicine at 12:00 PM.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -619,26 +592,21 @@
     "content": "What tasks do I have today"
   },
   {
-    "source": "agent",
-    "format": "audio",
-    "content": "One moment, let me check your tasks."
-  },
-  {
     "source": "agent_internal",
     "format": "function_call",
     "name": "get_tasks_tool",
     "response": {
-      "result": "{\"tasks\": [{\"task_id\": \"78f684f2-2180-4199-a280-2c5f23cc222a\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
+      "result": "{\"tasks\": [{\"task_id\": \"518cc49a-c8be-4c29-8e6a-50583dba906b\", \"user_id\": \"2ba330c0-a999-46f8-ba2c-855880bdcf5b\", \"task_info\": {\"info\": \"take my medicine\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T12:00:00-08:00\", \"enqueue_sequence_id\": null}], \"total_count\": 1}"
     },
-    "elapsed_s": 13.2
+    "elapsed_s": 10.72
   },
   {
     "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-12445068861386789067",
+    "call_id": "fc_6575505260845244972",
     "response": {
-      "result": "\n\n\nYou have one task scheduled for today:\n\n- take my medicine at 12:00 PM today."
+      "result": "You have one task scheduled for today: take my medicine at 12:00 PM."
     },
     "elapsed_s": 0.0
   },
@@ -668,7 +636,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-78f684f2-2180-4199-a280-2c5f23cc222a | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+518cc49a-c8be-4c29-8e6a-50583dba906b | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -686,7 +654,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-78f684f2-2180-4199-a280-2c5f23cc222a | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
+518cc49a-c8be-4c29-8e6a-50583dba906b | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'take my medicine'} | pending | 2026-03-01 12:00:00-08:00 | None
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>
@@ -705,7 +673,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>AGENT: One moment. I've scheduled a reminder for you to stretch at 10:00 PM today.</t>
+          <t>AGENT: Of course! I've set a reminder to stretch at 10:00 PM today.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -717,33 +685,28 @@
     "content": "Can you remind me to strecth at 10pm tonight?"
   },
   {
-    "source": "agent",
-    "format": "audio",
-    "content": "One moment."
-  },
-  {
     "source": "agent_internal",
     "format": "function_call",
     "name": "create_tasks_tool",
     "response": {
-      "result": "{\"success\": true, \"message\": \"Task '{'info': 'strecth'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"a7e7b8d2-f0b7-4007-8116-4dc1a3e4306f\", \"task_info\": {\"info\": \"strecth\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T22:00:00-08:00\"}"
+      "result": "{\"success\": true, \"message\": \"Task '{'info': 'stretch'}' created successfully. We don't need another create task tool call for this user instruction unless the user has asked for more tasks than this one you just created.\", \"task_id\": \"7265baa4-2fd8-4495-beba-57cdee2e1fbf\", \"task_info\": {\"info\": \"stretch\"}, \"status\": \"pending\", \"time_to_execute\": \"2026-03-01T22:00:00-08:00\"}"
     },
-    "elapsed_s": 14.39
+    "elapsed_s": 10.31
   },
   {
     "source": "agent",
     "format": "function_call",
     "name": "think_and_repeat_output",
-    "call_id": "function-call-17990089963753904540",
+    "call_id": "fc_15086125725975761893",
     "response": {
-      "result": "I've scheduled a reminder for you to strecth at 10:00 PM today."
+      "result": "\n\nOf course! I've set a reminder to stretch at 10:00 PM today."
     },
     "elapsed_s": 0.0
   },
   {
     "source": "agent",
     "format": "audio",
-    "content": "I've scheduled a reminder for you to stretch at 10:00 PM today."
+    "content": "Of course! I've set a reminder to stretch at 10:00 PM today."
   }
 ]</t>
         </is>
@@ -781,7 +744,7 @@
 [tasks]:
 task_id | user_id | task_info | status | time_to_execute | enqueue_sequence_id
 ------------------------------------------------------------------------------
-a7e7b8d2-f0b7-4007-8116-4dc1a3e4306f | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'strecth'} | pending | 2026-03-01 22:00:00-08:00 | None
+7265baa4-2fd8-4495-beba-57cdee2e1fbf | 2ba330c0-a999-46f8-ba2c-855880bdcf5b | {'info': 'stretch'} | pending | 2026-03-01 22:00:00-08:00 | None
 [messages]: (empty)
 [pending_text_message_jobs]: (empty)</t>
         </is>

</xml_diff>